<commit_message>
resolve timezone issue, native and tz-aware, also make sure that missed data is inserted in db
</commit_message>
<xml_diff>
--- a/symbols.xlsx
+++ b/symbols.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45518</v>
+        <v>45533</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45526</v>
+        <v>45540</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45533</v>
+        <v>45561</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45561</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="6">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45518</v>
+        <v>45532</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45525</v>
+        <v>45539</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45517</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45524</v>
+        <v>45538</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45516</v>
+        <v>45530</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45523</v>
+        <v>45537</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new and old app check
</commit_message>
<xml_diff>
--- a/symbols.xlsx
+++ b/symbols.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45518</v>
+        <v>45568</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45526</v>
+        <v>45575</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45533</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45561</v>
+        <v>45624</v>
       </c>
     </row>
     <row r="6">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45518</v>
+        <v>45566</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45525</v>
+        <v>45574</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45517</v>
+        <v>45566</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45524</v>
+        <v>45573</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45516</v>
+        <v>45572</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45523</v>
+        <v>45579</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added color to table
</commit_message>
<xml_diff>
--- a/symbols.xlsx
+++ b/symbols.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45533</v>
+        <v>45568</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45540</v>
+        <v>45575</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45561</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45596</v>
+        <v>45624</v>
       </c>
     </row>
     <row r="6">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45532</v>
+        <v>45574</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45539</v>
+        <v>45581</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45531</v>
+        <v>45573</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45538</v>
+        <v>45580</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45530</v>
+        <v>45572</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45537</v>
+        <v>45579</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added color in table
</commit_message>
<xml_diff>
--- a/symbols.xlsx
+++ b/symbols.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45568</v>
+        <v>45575</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45575</v>
+        <v>45582</v>
       </c>
     </row>
     <row r="4">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45566</v>
+        <v>45574</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45574</v>
+        <v>45581</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45566</v>
+        <v>45573</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45573</v>
+        <v>45580</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
weekly -> monthly expiry
</commit_message>
<xml_diff>
--- a/symbols.xlsx
+++ b/symbols.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45575</v>
+        <v>45624</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45582</v>
+        <v>45631</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45596</v>
+        <v>45652</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45624</v>
+        <v>45687</v>
       </c>
     </row>
     <row r="6">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45574</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45581</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45573</v>
+        <v>45657</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45580</v>
+        <v>45685</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45572</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45579</v>
+        <v>45684</v>
       </c>
     </row>
   </sheetData>

</xml_diff>